<commit_message>
Expand medium-scale study sampling plan
</commit_message>
<xml_diff>
--- a/outputs/goal2-research-registry-20260830/EVSP_DR_goal1_goal2_research_registry.xlsx
+++ b/outputs/goal2-research-registry-20260830/EVSP_DR_goal1_goal2_research_registry.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proof Summary" sheetId="1" r:id="R3a8f5507c62b4485"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" r:id="R81716b6c6b6448f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal1 Proofs" sheetId="3" r:id="R66b32cfa6b2d4116"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Proofs" sheetId="4" r:id="R657f14c137274a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal2 Instances" sheetId="5" r:id="Rfc867828478b4990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Ladder" sheetId="6" r:id="R52fb1c16f8f644f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sampling Plan" sheetId="7" r:id="R3527f0d9da0642f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Schema" sheetId="8" r:id="R0870f6451dba4ad2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proof Summary" sheetId="1" r:id="Rde509c862bdf41b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" r:id="Re32a8cb217794532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal1 Proofs" sheetId="3" r:id="Ra6733a7d37754b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Proofs" sheetId="4" r:id="R9d43c94d41d04d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Goal2 Instances" sheetId="5" r:id="Rf210135a8dee410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Ladder" sheetId="6" r:id="R3c59db0266e94dc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sampling Plan" sheetId="7" r:id="R8be3afdb96304fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Schema" sheetId="8" r:id="R44de96ba358145dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,7 +672,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a694a3207f4b02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R641f5f5c8e554179"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -777,7 +777,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dfe1ebbd2da459e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba6f639ee8c6477c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5807,7 +5807,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0ec266f96ac4f33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5ddb3724ba4549"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6236,7 +6236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b96783760e04dab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcffc9d20edfa497f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9680,7 +9680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d27c46e03194d18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R797a0ee374d9451f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12751,7 +12751,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c3ab66d97b841e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra41235f7094a43a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12766,8 +12766,8 @@
     <x:col min="4" max="4" width="19.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.779999732971191" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="66.77999877929688" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="39.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="71.66999816894531" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -12885,19 +12885,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D5" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E5" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="6" t="n">
-        <x:v>18</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
-        <x:v>new probability sample; legacy and stress rows separate</x:v>
+        <x:v>12-row probability sample; legacy and stress rows separate</x:v>
       </x:c>
       <x:c r="H5" s="6" t="str">
-        <x:v>fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
+        <x:v>staged fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -12911,19 +12911,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F6" s="6" t="n">
-        <x:v>12</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str">
-        <x:v>new probability sample; stress rows separate</x:v>
+        <x:v>12-row probability sample; stress rows separate</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
-        <x:v>fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
+        <x:v>staged fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -12937,19 +12937,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D7" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E7" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F7" s="6" t="n">
-        <x:v>18</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>new probability sample; legacy and stress rows separate</x:v>
+        <x:v>12-row probability sample; legacy and stress rows separate</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
+        <x:v>staged fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -12963,19 +12963,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="6" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E8" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="F8" s="6" t="n">
-        <x:v>18</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
-        <x:v>new probability sample; legacy and stress rows separate</x:v>
+        <x:v>12-row probability sample; legacy and stress rows separate</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
-        <x:v>fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
+        <x:v>staged fixed-seed random within trip-count x compatibility strata plus maximin feature-space stress sample</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -13033,7 +13033,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f0e63c920d64e3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rced436e53f8b4b9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13834,7 +13834,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4802d4ff0d54b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce89fa38e85c4e0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>